<commit_message>
Build: (d7dd09c) Add enemy info to game scene
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,65 +409,83 @@
       <c r="C1" t="str">
         <v>Experience</v>
       </c>
+      <c r="D1" t="str">
+        <v>Description</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Goblin</v>
-      </c>
-      <c r="B2">
+        <v>Chad the Mad</v>
+      </c>
+      <c r="B2" t="str">
         <v>300</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="str">
         <v>45</v>
+      </c>
+      <c r="D2" t="str">
+        <v>A hothead with anger issues and 300 HP.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Skeleton</v>
-      </c>
-      <c r="B3">
+        <v>Steven Invinsible</v>
+      </c>
+      <c r="B3" t="str">
         <v>450</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="str">
         <v>70</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Spells badly, fights well. Tough guy.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Orc</v>
-      </c>
-      <c r="B4">
+        <v>Manly O'Well</v>
+      </c>
+      <c r="B4" t="str">
         <v>700</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="str">
         <v>120</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Peak masculinity. Punches through steel.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Troll</v>
-      </c>
-      <c r="B5">
+        <v>Jessica Johannson</v>
+      </c>
+      <c r="B5" t="str">
         <v>1200</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="str">
         <v>220</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Deceptively cheery. Absolutely terrifying.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Dragon</v>
-      </c>
-      <c r="B6">
+        <v>Lil' Phil</v>
+      </c>
+      <c r="B6" t="str">
         <v>2500</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="str">
         <v>600</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Tiny body, colossal fury. 2500 HP. Run.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (b49f16b) Add some JUICE to battles
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,6 +412,9 @@
       <c r="D1" t="str">
         <v>Description</v>
       </c>
+      <c r="E1" t="str">
+        <v>Power</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -426,6 +429,9 @@
       <c r="D2" t="str">
         <v>A hothead with anger issues and 300 HP.</v>
       </c>
+      <c r="E2">
+        <v>18</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -440,6 +446,9 @@
       <c r="D3" t="str">
         <v>Spells badly, fights well. Tough guy.</v>
       </c>
+      <c r="E3">
+        <v>26</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -454,6 +463,9 @@
       <c r="D4" t="str">
         <v>Peak masculinity. Punches through steel.</v>
       </c>
+      <c r="E4">
+        <v>38</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -468,6 +480,9 @@
       <c r="D5" t="str">
         <v>Deceptively cheery. Absolutely terrifying.</v>
       </c>
+      <c r="E5">
+        <v>55</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -482,10 +497,13 @@
       <c r="D6" t="str">
         <v>Tiny body, colossal fury. 2500 HP. Run.</v>
       </c>
+      <c r="E6">
+        <v>90</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (23a83ae) Add walking animations to the enemies
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +415,9 @@
       <c r="E1" t="str">
         <v>Power</v>
       </c>
+      <c r="F1" t="str">
+        <v>Sprite</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -427,10 +430,13 @@
         <v>45</v>
       </c>
       <c r="D2" t="str">
-        <v>A hothead with anger issues and 300 HP.</v>
-      </c>
-      <c r="E2">
+        <v>"Boy howdy I am one incredibly angry dude!"</v>
+      </c>
+      <c r="E2" t="str">
         <v>18</v>
+      </c>
+      <c r="F2" t="str">
+        <v>sprites/Warrior.gif</v>
       </c>
     </row>
     <row r="3">
@@ -444,10 +450,13 @@
         <v>70</v>
       </c>
       <c r="D3" t="str">
-        <v>Spells badly, fights well. Tough guy.</v>
-      </c>
-      <c r="E3">
+        <v>"Ain't nothin' ganna kill me, I'm the strongast man who ever did done live dont'chuh know it"</v>
+      </c>
+      <c r="E3" t="str">
         <v>26</v>
+      </c>
+      <c r="F3" t="str">
+        <v>sprites/Mage.gif</v>
       </c>
     </row>
     <row r="4">
@@ -461,10 +470,13 @@
         <v>120</v>
       </c>
       <c r="D4" t="str">
-        <v>Peak masculinity. Punches through steel.</v>
-      </c>
-      <c r="E4">
+        <v>"Just wait until the boys hear about this one"</v>
+      </c>
+      <c r="E4" t="str">
         <v>38</v>
+      </c>
+      <c r="F4" t="str">
+        <v>sprites/Monk.gif</v>
       </c>
     </row>
     <row r="5">
@@ -478,10 +490,13 @@
         <v>220</v>
       </c>
       <c r="D5" t="str">
-        <v>Deceptively cheery. Absolutely terrifying.</v>
-      </c>
-      <c r="E5">
+        <v>" ... "</v>
+      </c>
+      <c r="E5" t="str">
         <v>55</v>
+      </c>
+      <c r="F5" t="str">
+        <v>sprites/Thief.gif</v>
       </c>
     </row>
     <row r="6">
@@ -495,15 +510,18 @@
         <v>600</v>
       </c>
       <c r="D6" t="str">
-        <v>Tiny body, colossal fury. 2500 HP. Run.</v>
-      </c>
-      <c r="E6">
+        <v>"Who you callin' little?!"</v>
+      </c>
+      <c r="E6" t="str">
         <v>90</v>
+      </c>
+      <c r="F6" t="str">
+        <v>sprites/Warrior.gif</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (727fb34) Small QOL changes
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -436,7 +436,7 @@
         <v>45</v>
       </c>
       <c r="D2" t="str">
-        <v>"Boy howdy I am one incredibly angry dude!"</v>
+        <v>"Boy howdy am I ANGRY!!!"</v>
       </c>
       <c r="E2" t="str">
         <v>18</v>
@@ -450,7 +450,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Steven Invinsible</v>
+        <v>Steven Invincible</v>
       </c>
       <c r="B3" t="str">
         <v>450</v>
@@ -459,7 +459,7 @@
         <v>70</v>
       </c>
       <c r="D3" t="str">
-        <v>"Ain't nothin' ganna kill me, I'm the strongast man who ever did done live dont'chuh know it"</v>
+        <v>"Keep your head down Steven. Move forward. They can't hurt you... They can't hurt you..."</v>
       </c>
       <c r="E3" t="str">
         <v>26</v>

</xml_diff>

<commit_message>
Build: (6ca343a) Finalizing the current layout
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:K6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,6 +424,15 @@
       <c r="H1" t="str">
         <v>Weak2</v>
       </c>
+      <c r="I1" t="str">
+        <v>Element1</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Element2</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Element3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -447,6 +456,12 @@
       <c r="G2" t="str">
         <v>Fire</v>
       </c>
+      <c r="I2" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="J2" t="str">
+        <v>💧</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -542,7 +557,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (12026dd) Final touches
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -474,7 +474,7 @@
         <v>70</v>
       </c>
       <c r="D3" t="str">
-        <v>"Keep your head down Steven. Move forward. They can't hurt you... They can't hurt you..."</v>
+        <v>"I'M INVINCIBLE!!"</v>
       </c>
       <c r="E3" t="str">
         <v>26</v>
@@ -497,7 +497,7 @@
         <v>120</v>
       </c>
       <c r="D4" t="str">
-        <v>"Just wait until the boys hear about this one"</v>
+        <v>"I'll give 'em the ol' One-Two Puncharoo"</v>
       </c>
       <c r="E4" t="str">
         <v>38</v>

</xml_diff>

<commit_message>
Build: (ae8516b) Add elements to all enemies
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -457,9 +457,6 @@
         <v>Fire</v>
       </c>
       <c r="I2" t="str">
-        <v>🔥</v>
-      </c>
-      <c r="J2" t="str">
         <v>💧</v>
       </c>
     </row>
@@ -483,7 +480,10 @@
         <v>sprites/Mage.gif</v>
       </c>
       <c r="G3" t="str">
-        <v>Water</v>
+        <v>Earth</v>
+      </c>
+      <c r="I3" t="str">
+        <v>⚡</v>
       </c>
     </row>
     <row r="4">
@@ -508,6 +508,9 @@
       <c r="G4" t="str">
         <v>Lightning</v>
       </c>
+      <c r="I4" t="str">
+        <v>🍃</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -529,7 +532,10 @@
         <v>sprites/Thief.gif</v>
       </c>
       <c r="G5" t="str">
-        <v>Earth</v>
+        <v>Water</v>
+      </c>
+      <c r="I5" t="str">
+        <v>🔥</v>
       </c>
     </row>
     <row r="6">
@@ -553,6 +559,12 @@
       </c>
       <c r="G6" t="str">
         <v>Steel</v>
+      </c>
+      <c r="I6" t="str">
+        <v>💧</v>
+      </c>
+      <c r="J6" t="str">
+        <v>⚡</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Build: (617b61f) Fix icon sizes in fight
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -438,10 +438,10 @@
       <c r="A2" t="str">
         <v>Chad the Mad</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="str">
         <v>75</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="str">
         <v>40</v>
       </c>
       <c r="D2" t="str">
@@ -460,7 +460,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>💧</v>
+        <v>Water</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -473,10 +473,10 @@
       <c r="A3" t="str">
         <v>Steven Invincible</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="str">
         <v>140</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="str">
         <v>65</v>
       </c>
       <c r="D3" t="str">
@@ -508,10 +508,10 @@
       <c r="A4" t="str">
         <v>Manly O'Well</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="str">
         <v>180</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="str">
         <v>100</v>
       </c>
       <c r="D4" t="str">
@@ -543,10 +543,10 @@
       <c r="A5" t="str">
         <v>Jessica Johannson</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="str">
         <v>240</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="str">
         <v>170</v>
       </c>
       <c r="D5" t="str">
@@ -578,10 +578,10 @@
       <c r="A6" t="str">
         <v>Lil' Phil</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="str">
         <v>360</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="str">
         <v>300</v>
       </c>
       <c r="D6" t="str">

</xml_diff>

<commit_message>
Build: (8610538) Balance update. Bug fix: level 2 elements were combining. Minor QoL updates.
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -454,19 +454,16 @@
         <v>sprites/Warrior.gif</v>
       </c>
       <c r="G2" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>Water</v>
-      </c>
-      <c r="J2" t="str">
         <v>Fire</v>
       </c>
       <c r="K2" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -495,13 +492,10 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>Water Bolt</v>
+        <v>Water</v>
       </c>
       <c r="J3" t="str">
-        <v>Tornado</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Thorns</v>
+        <v>Worble</v>
       </c>
     </row>
     <row r="4">
@@ -524,19 +518,16 @@
         <v>sprites/Monk.gif</v>
       </c>
       <c r="G4" t="str">
-        <v>Lightning</v>
+        <v>Fire</v>
       </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>Ice Shield</v>
+        <v>Ice</v>
       </c>
       <c r="J4" t="str">
-        <v>Blaze Blade</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Thunder</v>
+        <v>Glacier</v>
       </c>
     </row>
     <row r="5">
@@ -567,12 +558,6 @@
       <c r="I5" t="str">
         <v>Pyreball</v>
       </c>
-      <c r="J5" t="str">
-        <v>Glacier</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Leaf Blade</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -594,19 +579,13 @@
         <v>sprites/Warrior.gif</v>
       </c>
       <c r="G6" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
         <v>Thunder</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Earthquake</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Refined Steel</v>
       </c>
     </row>
   </sheetData>

</xml_diff>